<commit_message>
chore: fix path length issues and update test specs
</commit_message>
<xml_diff>
--- a/cypress/downloads/BAS_Client_Template.xlsx
+++ b/cypress/downloads/BAS_Client_Template.xlsx
@@ -19,16 +19,16 @@
     <x:t>FirstName*</x:t>
   </x:si>
   <x:si>
-    <x:t>LastName</x:t>
+    <x:t>LastName*</x:t>
   </x:si>
   <x:si>
     <x:t>PhoneNumber*</x:t>
   </x:si>
   <x:si>
-    <x:t>Email</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Address</x:t>
+    <x:t>Email*</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Address*</x:t>
   </x:si>
   <x:si>
     <x:t>DateOfBirth (yyyy-MM-dd)</x:t>
@@ -430,7 +430,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="10.996339" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="9.710625" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10.710625" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="15.139196" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="23.282054" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="26.567768" style="0" customWidth="1"/>

</xml_diff>

<commit_message>
creating at onboarding added and UI changes
</commit_message>
<xml_diff>
--- a/cypress/downloads/BAS_Client_Template.xlsx
+++ b/cypress/downloads/BAS_Client_Template.xlsx
@@ -77,7 +77,7 @@
       <x:b/>
       <x:vertAlign val="baseline"/>
       <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
+      <x:color rgb="FFFFFFFF"/>
       <x:name val="Calibri"/>
       <x:family val="2"/>
     </x:font>
@@ -91,7 +91,7 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFD3D3D3"/>
+        <x:fgColor rgb="FF0F766E"/>
       </x:patternFill>
     </x:fill>
   </x:fills>

</xml_diff>